<commit_message>
Fix invoice review, cash signs, Excel amounts, and deploy safety.
Hardened create/review flows for LAN servers: signed cash warehouse by transaction type, portable Excel paths, merged DB migrations, and Gradio wiring so dashboard data shows reliably after pull.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/templates/invoice_template.xlsx
+++ b/templates/invoice_template.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="693" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="銷售" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="購入單" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="兌料單" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="交收單" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="銷售" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="購入單" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="兌料單" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="交收單" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'銷售'!$A$1:$K$54</definedName>
@@ -718,7 +718,7 @@
       <c r="J8" s="30" t="n"/>
       <c r="K8" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">金額 </t>
+          <t>現金倉</t>
         </is>
       </c>
     </row>
@@ -749,7 +749,7 @@
       <c r="J9" s="30" t="n"/>
       <c r="K9" s="30" t="inlineStr">
         <is>
-          <t>Amount</t>
+          <t>Cash Warehouse</t>
         </is>
       </c>
     </row>
@@ -1132,7 +1132,7 @@
       </c>
       <c r="J35" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">金額 </t>
+          <t>現金倉</t>
         </is>
       </c>
     </row>
@@ -1165,7 +1165,7 @@
       </c>
       <c r="J36" s="30" t="inlineStr">
         <is>
-          <t>Amount</t>
+          <t>Cash Warehouse</t>
         </is>
       </c>
     </row>
@@ -1555,7 +1555,7 @@
       <c r="J8" s="30" t="n"/>
       <c r="K8" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">金額 </t>
+          <t>現金倉</t>
         </is>
       </c>
     </row>
@@ -1586,7 +1586,7 @@
       <c r="J9" s="30" t="n"/>
       <c r="K9" s="30" t="inlineStr">
         <is>
-          <t>Amount</t>
+          <t>Cash Warehouse</t>
         </is>
       </c>
     </row>
@@ -1985,7 +1985,7 @@
       </c>
       <c r="J35" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">金額 </t>
+          <t>現金倉</t>
         </is>
       </c>
     </row>
@@ -2018,7 +2018,7 @@
       </c>
       <c r="J36" s="30" t="inlineStr">
         <is>
-          <t>Amount</t>
+          <t>Cash Warehouse</t>
         </is>
       </c>
     </row>
@@ -2460,7 +2460,7 @@
       <c r="J8" s="30" t="n"/>
       <c r="K8" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">金額 </t>
+          <t>現金倉</t>
         </is>
       </c>
     </row>
@@ -2491,7 +2491,7 @@
       <c r="J9" s="30" t="n"/>
       <c r="K9" s="30" t="inlineStr">
         <is>
-          <t>Amount</t>
+          <t>Cash Warehouse</t>
         </is>
       </c>
     </row>
@@ -2865,7 +2865,7 @@
       </c>
       <c r="J35" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">金額 </t>
+          <t>現金倉</t>
         </is>
       </c>
     </row>
@@ -2900,7 +2900,7 @@
       </c>
       <c r="J36" s="30" t="inlineStr">
         <is>
-          <t>Amount</t>
+          <t>Cash Warehouse</t>
         </is>
       </c>
     </row>
@@ -3359,7 +3359,7 @@
       <c r="J8" s="30" t="n"/>
       <c r="K8" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">金額 </t>
+          <t>現金倉</t>
         </is>
       </c>
     </row>
@@ -3390,7 +3390,7 @@
       <c r="J9" s="30" t="n"/>
       <c r="K9" s="30" t="inlineStr">
         <is>
-          <t>Amount</t>
+          <t>Cash Warehouse</t>
         </is>
       </c>
     </row>
@@ -3725,7 +3725,7 @@
       </c>
       <c r="J35" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">金額 </t>
+          <t>現金倉</t>
         </is>
       </c>
     </row>
@@ -3760,7 +3760,7 @@
       </c>
       <c r="J36" s="30" t="inlineStr">
         <is>
-          <t>Amount</t>
+          <t>Cash Warehouse</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ship Perfect V2 receipt PDF, Excel-backed preview, and inventory auto-refresh.
Remove hard-coded stock labels from Excel/PDF print path; refresh warehouse totals after invoice generate.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/templates/invoice_template.xlsx
+++ b/templates/invoice_template.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="693" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="銷售" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="購入單" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="兌料單" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="交收單" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="銷售" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="購入單" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="兌料單" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="交收單" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'銷售'!$A$1:$K$54</definedName>
@@ -651,8 +651,8 @@
     <col width="13.5" customWidth="1" style="30" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" ht="45" customHeight="1" s="36"/>
-    <row r="2" ht="42" customHeight="1" s="36">
+    <row r="1" ht="50" customHeight="1" s="36"/>
+    <row r="2" ht="45" customHeight="1" s="36">
       <c r="K2" s="28" t="n"/>
     </row>
     <row r="3" ht="10" customHeight="1" s="36">
@@ -1063,8 +1063,8 @@
       <c r="J27" s="30" t="n"/>
       <c r="K27" s="30" t="n"/>
     </row>
-    <row r="28" ht="34" customHeight="1" s="36"/>
-    <row r="29" ht="32" customHeight="1" s="36"/>
+    <row r="28" ht="38" customHeight="1" s="36"/>
+    <row r="29" ht="34" customHeight="1" s="36"/>
     <row r="30" ht="10" customHeight="1" s="36">
       <c r="K30" s="28" t="n"/>
     </row>
@@ -1488,8 +1488,8 @@
     <col width="13.5" customWidth="1" style="30" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" ht="45" customHeight="1" s="36"/>
-    <row r="2" ht="42" customHeight="1" s="36">
+    <row r="1" ht="50" customHeight="1" s="36"/>
+    <row r="2" ht="45" customHeight="1" s="36">
       <c r="K2" s="28" t="n"/>
     </row>
     <row r="3" ht="10" customHeight="1" s="36">
@@ -1916,8 +1916,8 @@
       <c r="J27" s="30" t="n"/>
       <c r="K27" s="30" t="n"/>
     </row>
-    <row r="28" ht="34" customHeight="1" s="36"/>
-    <row r="29" ht="32" customHeight="1" s="36"/>
+    <row r="28" ht="38" customHeight="1" s="36"/>
+    <row r="29" ht="34" customHeight="1" s="36"/>
     <row r="30" ht="10" customHeight="1" s="36">
       <c r="K30" s="28" t="n"/>
     </row>
@@ -2393,8 +2393,8 @@
     <col width="13.5" customWidth="1" style="30" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" ht="45" customHeight="1" s="36"/>
-    <row r="2" ht="42" customHeight="1" s="36">
+    <row r="1" ht="50" customHeight="1" s="36"/>
+    <row r="2" ht="45" customHeight="1" s="36">
       <c r="K2" s="28" t="n"/>
     </row>
     <row r="3" ht="10" customHeight="1" s="36">
@@ -2794,8 +2794,8 @@
       <c r="J27" s="30" t="n"/>
       <c r="K27" s="30" t="n"/>
     </row>
-    <row r="28" ht="34" customHeight="1" s="36"/>
-    <row r="29" ht="32" customHeight="1" s="36"/>
+    <row r="28" ht="38" customHeight="1" s="36"/>
+    <row r="29" ht="34" customHeight="1" s="36"/>
     <row r="30" ht="10" customHeight="1" s="36">
       <c r="K30" s="28" t="n"/>
     </row>
@@ -3292,8 +3292,8 @@
     <col width="13.5" customWidth="1" style="30" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" ht="45" customHeight="1" s="36"/>
-    <row r="2" ht="42" customHeight="1" s="36">
+    <row r="1" ht="50" customHeight="1" s="36"/>
+    <row r="2" ht="45" customHeight="1" s="36">
       <c r="K2" s="28" t="n"/>
     </row>
     <row r="3" ht="10" customHeight="1" s="36">
@@ -3654,8 +3654,8 @@
       <c r="J27" s="30" t="n"/>
       <c r="K27" s="30" t="n"/>
     </row>
-    <row r="28" ht="34" customHeight="1" s="36"/>
-    <row r="29" ht="32" customHeight="1" s="36"/>
+    <row r="28" ht="38" customHeight="1" s="36"/>
+    <row r="29" ht="34" customHeight="1" s="36"/>
     <row r="30" ht="10" customHeight="1" s="36">
       <c r="K30" s="28" t="n"/>
     </row>

</xml_diff>